<commit_message>
Add unscored vendor-direction context to intake.
Questionnaire 1.1.0 records vendor direction, residual direction, and a short note for a reviewer. The risk engine does not read those fields, so the residual tier and disposition stay the same when the context changes.

Co-authored-by: doneal78 <doneal78@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/imports/vendor_intake.xlsx
+++ b/tests/fixtures/imports/vendor_intake.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,21 @@
           <t>evidence_clause_CC-001</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>vendor_direction</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>residual_direction</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>direction_note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -559,6 +574,21 @@
           <t>independent_verified</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>unchanged</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Synthetic context: same scope as the last review. Not a score.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -625,6 +655,21 @@
       <c r="N3" t="inlineStr">
         <is>
           <t>vendor_statement</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>expanding</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>worsening</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Synthetic context: more use than the last review. Not a score.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add unscored vendor-direction context to intake (#20)
Optional vendor_direction, residual_direction, and direction_note as reviewer context. Residual formula and scoring unchanged.
</commit_message>
<xml_diff>
--- a/tests/fixtures/imports/vendor_intake.xlsx
+++ b/tests/fixtures/imports/vendor_intake.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,21 @@
           <t>evidence_clause_CC-001</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>vendor_direction</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>residual_direction</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>direction_note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -559,6 +574,21 @@
           <t>independent_verified</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>unchanged</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Synthetic context: same scope as the last review. Not a score.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -625,6 +655,21 @@
       <c r="N3" t="inlineStr">
         <is>
           <t>vendor_statement</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>expanding</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>worsening</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Synthetic context: more use than the last review. Not a score.</t>
         </is>
       </c>
     </row>

</xml_diff>